<commit_message>
Agregar módulo Agua Tratada
</commit_message>
<xml_diff>
--- a/assets/templates/reporte-diario-agua-tratada.xlsx
+++ b/assets/templates/reporte-diario-agua-tratada.xlsx
@@ -700,88 +700,158 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="10" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="20" fontId="10" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="2" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="11" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="11" fillId="4" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="11" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="2" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="1" fillId="2" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="3" fontId="1" fillId="2" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="11" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="11" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="1" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="1" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="1" fillId="2" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="1" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -791,80 +861,8 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="1" fillId="2" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="1" fillId="2" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="1" fillId="2" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="11" fillId="4" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="10" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="10" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1581,7 +1579,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9EA1F24-8A5A-4511-9238-ABA1E84E1E22}">
-  <dimension ref="A1:Q30"/>
+  <dimension ref="A1:P30"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="4.25" customWidth="1"/>
@@ -1597,579 +1595,542 @@
     <col min="15" max="15" width="17.375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="14.25" customHeight="1">
-      <c r="A1" s="8" t="s">
+    <row r="1" spans="1:16" ht="14.25" customHeight="1">
+      <c r="A1" s="39" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
-      <c r="H1" s="8"/>
-      <c r="I1" s="8"/>
-      <c r="J1" s="8"/>
-      <c r="K1" s="8"/>
-      <c r="L1" s="8"/>
-      <c r="M1" s="8"/>
-      <c r="N1" s="8"/>
-      <c r="O1" s="8"/>
-    </row>
-    <row r="2" spans="1:17" ht="14.25" customHeight="1">
-      <c r="A2" s="8"/>
-      <c r="B2" s="8"/>
-      <c r="C2" s="8"/>
-      <c r="D2" s="8"/>
-      <c r="E2" s="8"/>
-      <c r="F2" s="8"/>
-      <c r="G2" s="8"/>
-      <c r="H2" s="8"/>
-      <c r="I2" s="8"/>
-      <c r="J2" s="8"/>
-      <c r="K2" s="8"/>
-      <c r="L2" s="8"/>
-      <c r="M2" s="8"/>
-      <c r="N2" s="8"/>
-      <c r="O2" s="8"/>
-    </row>
-    <row r="3" spans="1:17" ht="14.25" customHeight="1">
-      <c r="A3" s="8"/>
-      <c r="B3" s="8"/>
-      <c r="C3" s="8"/>
-      <c r="D3" s="8"/>
-      <c r="E3" s="8"/>
-      <c r="F3" s="8"/>
-      <c r="G3" s="8"/>
-      <c r="H3" s="8"/>
-      <c r="I3" s="8"/>
-      <c r="J3" s="8"/>
-      <c r="K3" s="8"/>
-      <c r="L3" s="8"/>
-      <c r="M3" s="8"/>
-      <c r="N3" s="8"/>
-      <c r="O3" s="8"/>
-    </row>
-    <row r="4" spans="1:17" ht="14.25" customHeight="1">
-      <c r="A4" s="5"/>
-      <c r="B4" s="5"/>
-      <c r="C4" s="5"/>
-      <c r="D4" s="9" t="s">
+      <c r="B1" s="39"/>
+      <c r="C1" s="39"/>
+      <c r="D1" s="39"/>
+      <c r="E1" s="39"/>
+      <c r="F1" s="39"/>
+      <c r="G1" s="39"/>
+      <c r="H1" s="39"/>
+      <c r="I1" s="39"/>
+      <c r="J1" s="39"/>
+      <c r="K1" s="39"/>
+      <c r="L1" s="39"/>
+      <c r="M1" s="39"/>
+      <c r="N1" s="39"/>
+      <c r="O1" s="39"/>
+    </row>
+    <row r="2" spans="1:16" ht="14.25" customHeight="1">
+      <c r="A2" s="39"/>
+      <c r="B2" s="39"/>
+      <c r="C2" s="39"/>
+      <c r="D2" s="39"/>
+      <c r="E2" s="39"/>
+      <c r="F2" s="39"/>
+      <c r="G2" s="39"/>
+      <c r="H2" s="39"/>
+      <c r="I2" s="39"/>
+      <c r="J2" s="39"/>
+      <c r="K2" s="39"/>
+      <c r="L2" s="39"/>
+      <c r="M2" s="39"/>
+      <c r="N2" s="39"/>
+      <c r="O2" s="39"/>
+    </row>
+    <row r="3" spans="1:16" ht="14.25" customHeight="1">
+      <c r="A3" s="39"/>
+      <c r="B3" s="39"/>
+      <c r="C3" s="39"/>
+      <c r="D3" s="39"/>
+      <c r="E3" s="39"/>
+      <c r="F3" s="39"/>
+      <c r="G3" s="39"/>
+      <c r="H3" s="39"/>
+      <c r="I3" s="39"/>
+      <c r="J3" s="39"/>
+      <c r="K3" s="39"/>
+      <c r="L3" s="39"/>
+      <c r="M3" s="39"/>
+      <c r="N3" s="39"/>
+      <c r="O3" s="39"/>
+    </row>
+    <row r="4" spans="1:16" ht="14.25" customHeight="1">
+      <c r="D4" s="40" t="s">
         <v>1</v>
       </c>
-      <c r="E4" s="9"/>
-      <c r="F4" s="9"/>
-      <c r="G4" s="9"/>
-      <c r="H4" s="9"/>
-      <c r="I4" s="9"/>
-      <c r="J4" s="9"/>
-      <c r="K4" s="9"/>
-      <c r="L4" s="9"/>
-      <c r="M4" s="5"/>
-    </row>
-    <row r="5" spans="1:17" ht="14.25" customHeight="1">
-      <c r="A5" s="5"/>
-      <c r="B5" s="5"/>
-      <c r="C5" s="5"/>
-      <c r="D5" s="9"/>
-      <c r="E5" s="9"/>
-      <c r="F5" s="9"/>
-      <c r="G5" s="9"/>
-      <c r="H5" s="9"/>
-      <c r="I5" s="9"/>
-      <c r="J5" s="9"/>
-      <c r="K5" s="9"/>
-      <c r="L5" s="9"/>
-      <c r="M5" s="5"/>
-    </row>
-    <row r="6" spans="1:17" ht="15" thickBot="1">
-      <c r="A6" s="6"/>
-      <c r="B6" s="6"/>
-      <c r="C6" s="6"/>
-      <c r="D6" s="6"/>
-      <c r="E6" s="6"/>
-      <c r="F6" s="6"/>
-      <c r="G6" s="6"/>
-      <c r="H6" s="6"/>
-      <c r="I6" s="6"/>
-      <c r="J6" s="6"/>
-      <c r="K6" s="6"/>
-      <c r="L6" s="6"/>
-      <c r="M6" s="14"/>
-      <c r="N6" s="14"/>
-      <c r="O6" s="14"/>
-      <c r="P6" s="6"/>
-    </row>
-    <row r="7" spans="1:17">
-      <c r="A7" s="13"/>
-      <c r="B7" s="13"/>
-      <c r="C7" s="13"/>
-      <c r="D7" s="13"/>
-      <c r="E7" s="13"/>
-      <c r="F7" s="13"/>
-      <c r="G7" s="13"/>
-      <c r="H7" s="13"/>
-      <c r="I7" s="13"/>
-      <c r="J7" s="13"/>
-      <c r="K7" s="13"/>
-      <c r="L7" s="13"/>
-      <c r="M7" s="5"/>
-      <c r="N7" s="5"/>
-    </row>
-    <row r="8" spans="1:17" ht="15">
-      <c r="B8" s="11" t="s">
+      <c r="E4" s="40"/>
+      <c r="F4" s="40"/>
+      <c r="G4" s="40"/>
+      <c r="H4" s="40"/>
+      <c r="I4" s="40"/>
+      <c r="J4" s="40"/>
+      <c r="K4" s="40"/>
+      <c r="L4" s="40"/>
+    </row>
+    <row r="5" spans="1:16" ht="14.25" customHeight="1">
+      <c r="D5" s="40"/>
+      <c r="E5" s="40"/>
+      <c r="F5" s="40"/>
+      <c r="G5" s="40"/>
+      <c r="H5" s="40"/>
+      <c r="I5" s="40"/>
+      <c r="J5" s="40"/>
+      <c r="K5" s="40"/>
+      <c r="L5" s="40"/>
+    </row>
+    <row r="6" spans="1:16" ht="15" thickBot="1">
+      <c r="A6" s="1"/>
+      <c r="B6" s="1"/>
+      <c r="C6" s="1"/>
+      <c r="D6" s="1"/>
+      <c r="E6" s="1"/>
+      <c r="F6" s="1"/>
+      <c r="G6" s="1"/>
+      <c r="H6" s="1"/>
+      <c r="I6" s="1"/>
+      <c r="J6" s="1"/>
+      <c r="K6" s="1"/>
+      <c r="L6" s="1"/>
+      <c r="M6" s="1"/>
+      <c r="N6" s="1"/>
+      <c r="O6" s="1"/>
+      <c r="P6" s="1"/>
+    </row>
+    <row r="7" spans="1:16">
+      <c r="A7" s="2"/>
+      <c r="B7" s="2"/>
+      <c r="C7" s="2"/>
+      <c r="D7" s="2"/>
+      <c r="E7" s="2"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
+      <c r="H7" s="2"/>
+      <c r="I7" s="2"/>
+      <c r="J7" s="2"/>
+      <c r="K7" s="2"/>
+      <c r="L7" s="2"/>
+    </row>
+    <row r="8" spans="1:16" ht="15">
+      <c r="B8" s="25" t="s">
         <v>18</v>
       </c>
-      <c r="C8" s="12"/>
-      <c r="D8" s="12"/>
-      <c r="E8" s="12"/>
-      <c r="F8" s="12"/>
-      <c r="G8" s="12"/>
-      <c r="H8" s="12"/>
-      <c r="I8" s="12"/>
-      <c r="J8" s="12"/>
-      <c r="K8" s="12"/>
-      <c r="L8" s="12"/>
-      <c r="M8" s="12"/>
-      <c r="N8" s="12"/>
-    </row>
-    <row r="10" spans="1:17" ht="30" customHeight="1">
-      <c r="B10" s="31" t="s">
+      <c r="C8" s="54"/>
+      <c r="D8" s="54"/>
+      <c r="E8" s="54"/>
+      <c r="F8" s="54"/>
+      <c r="G8" s="54"/>
+      <c r="H8" s="54"/>
+      <c r="I8" s="54"/>
+      <c r="J8" s="54"/>
+      <c r="K8" s="54"/>
+      <c r="L8" s="54"/>
+      <c r="M8" s="54"/>
+      <c r="N8" s="54"/>
+    </row>
+    <row r="10" spans="1:16" ht="30" customHeight="1">
+      <c r="B10" s="55" t="s">
         <v>2</v>
       </c>
-      <c r="C10" s="32"/>
-      <c r="D10" s="33" t="s">
+      <c r="C10" s="56"/>
+      <c r="D10" s="57" t="s">
         <v>19</v>
       </c>
-      <c r="E10" s="32"/>
-      <c r="F10" s="34" t="s">
+      <c r="E10" s="56"/>
+      <c r="F10" s="26" t="s">
         <v>20</v>
       </c>
-      <c r="G10" s="35"/>
-      <c r="H10" s="33" t="s">
+      <c r="G10" s="52"/>
+      <c r="H10" s="57" t="s">
         <v>23</v>
       </c>
-      <c r="I10" s="32"/>
-      <c r="J10" s="34" t="s">
+      <c r="I10" s="56"/>
+      <c r="J10" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="K10" s="36"/>
-      <c r="L10" s="34" t="s">
+      <c r="K10" s="58"/>
+      <c r="L10" s="26" t="s">
         <v>24</v>
       </c>
-      <c r="M10" s="35"/>
-      <c r="N10" s="34" t="s">
+      <c r="M10" s="52"/>
+      <c r="N10" s="26" t="s">
         <v>24</v>
       </c>
-      <c r="O10" s="37"/>
-    </row>
-    <row r="11" spans="1:17" ht="15">
-      <c r="B11" s="38" t="s">
+      <c r="O10" s="27"/>
+    </row>
+    <row r="11" spans="1:16" ht="15">
+      <c r="B11" s="53" t="s">
         <v>3</v>
       </c>
-      <c r="C11" s="4"/>
-      <c r="D11" s="15">
+      <c r="C11" s="35"/>
+      <c r="D11" s="36">
         <v>0</v>
       </c>
-      <c r="E11" s="15"/>
-      <c r="F11" s="15">
+      <c r="E11" s="36"/>
+      <c r="F11" s="36">
         <v>0</v>
       </c>
-      <c r="G11" s="15"/>
-      <c r="H11" s="15">
+      <c r="G11" s="36"/>
+      <c r="H11" s="36">
         <v>0</v>
       </c>
-      <c r="I11" s="15"/>
-      <c r="J11" s="15">
+      <c r="I11" s="36"/>
+      <c r="J11" s="36">
         <v>0</v>
       </c>
-      <c r="K11" s="15"/>
-      <c r="L11" s="15">
+      <c r="K11" s="36"/>
+      <c r="L11" s="36">
         <v>0</v>
       </c>
-      <c r="M11" s="15"/>
-      <c r="N11" s="15">
+      <c r="M11" s="36"/>
+      <c r="N11" s="36">
         <f>+D11+F11+H11-J11-L11</f>
         <v>0</v>
       </c>
-      <c r="O11" s="39"/>
-      <c r="Q11" s="5"/>
-    </row>
-    <row r="12" spans="1:17" ht="15">
-      <c r="B12" s="40" t="s">
+      <c r="O11" s="48"/>
+    </row>
+    <row r="12" spans="1:16" ht="15">
+      <c r="B12" s="50" t="s">
         <v>4</v>
       </c>
-      <c r="C12" s="41"/>
-      <c r="D12" s="42">
+      <c r="C12" s="51"/>
+      <c r="D12" s="47">
         <v>2000</v>
       </c>
-      <c r="E12" s="42"/>
-      <c r="F12" s="42">
+      <c r="E12" s="47"/>
+      <c r="F12" s="47">
         <v>0</v>
       </c>
-      <c r="G12" s="42"/>
-      <c r="H12" s="42">
+      <c r="G12" s="47"/>
+      <c r="H12" s="47">
         <v>0</v>
       </c>
-      <c r="I12" s="42"/>
-      <c r="J12" s="42">
+      <c r="I12" s="47"/>
+      <c r="J12" s="47">
         <v>800</v>
       </c>
-      <c r="K12" s="42"/>
-      <c r="L12" s="42">
+      <c r="K12" s="47"/>
+      <c r="L12" s="47">
         <v>0</v>
       </c>
-      <c r="M12" s="42"/>
-      <c r="N12" s="42">
+      <c r="M12" s="47"/>
+      <c r="N12" s="47">
         <f>+D12+F12+H12-J12-L12</f>
         <v>1200</v>
       </c>
-      <c r="O12" s="43"/>
-      <c r="Q12" s="5"/>
-    </row>
-    <row r="15" spans="1:17" ht="23.25">
-      <c r="B15" s="10" t="s">
+      <c r="O12" s="49"/>
+    </row>
+    <row r="15" spans="1:16" ht="23.25">
+      <c r="B15" s="24" t="s">
         <v>22</v>
       </c>
-      <c r="C15" s="10"/>
-      <c r="D15" s="10"/>
-      <c r="E15" s="10"/>
-      <c r="G15" s="16" t="s">
+      <c r="C15" s="24"/>
+      <c r="D15" s="24"/>
+      <c r="E15" s="24"/>
+      <c r="G15" s="43" t="s">
         <v>26</v>
       </c>
-      <c r="H15" s="7"/>
-      <c r="I15" s="7"/>
-      <c r="J15" s="7"/>
-      <c r="L15" s="17"/>
-      <c r="M15" s="11" t="s">
+      <c r="H15" s="44"/>
+      <c r="I15" s="44"/>
+      <c r="J15" s="44"/>
+      <c r="L15" s="3"/>
+      <c r="M15" s="25" t="s">
         <v>27</v>
       </c>
-      <c r="N15" s="10"/>
-      <c r="O15" s="10"/>
-      <c r="P15" s="10"/>
-    </row>
-    <row r="16" spans="1:17" ht="15">
-      <c r="G16" s="30"/>
-      <c r="H16" s="30"/>
-      <c r="I16" s="30"/>
-      <c r="J16" s="30"/>
-      <c r="K16" s="30"/>
-      <c r="L16" s="17"/>
-      <c r="M16" s="30"/>
-      <c r="N16" s="30"/>
-      <c r="O16" s="30"/>
+      <c r="N15" s="24"/>
+      <c r="O15" s="24"/>
+      <c r="P15" s="24"/>
+    </row>
+    <row r="16" spans="1:16" ht="15">
+      <c r="G16" s="6"/>
+      <c r="H16" s="6"/>
+      <c r="I16" s="6"/>
+      <c r="J16" s="6"/>
+      <c r="K16" s="6"/>
+      <c r="L16" s="3"/>
+      <c r="M16" s="6"/>
+      <c r="N16" s="6"/>
+      <c r="O16" s="6"/>
     </row>
     <row r="17" spans="2:15" ht="27" customHeight="1">
-      <c r="B17" s="1" t="s">
+      <c r="B17" s="41" t="s">
         <v>5</v>
       </c>
-      <c r="C17" s="2"/>
-      <c r="D17" s="1" t="s">
+      <c r="C17" s="42"/>
+      <c r="D17" s="41" t="s">
         <v>25</v>
       </c>
-      <c r="E17" s="2"/>
-      <c r="F17" s="45"/>
-      <c r="G17" s="28" t="s">
+      <c r="E17" s="42"/>
+      <c r="F17" s="8"/>
+      <c r="G17" s="45" t="s">
         <v>6</v>
       </c>
-      <c r="H17" s="28"/>
-      <c r="I17" s="29"/>
-      <c r="J17" s="34" t="s">
+      <c r="H17" s="45"/>
+      <c r="I17" s="46"/>
+      <c r="J17" s="26" t="s">
         <v>25</v>
       </c>
-      <c r="K17" s="37"/>
-      <c r="L17" s="5"/>
-      <c r="M17" s="46" t="s">
+      <c r="K17" s="27"/>
+      <c r="M17" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="N17" s="46" t="s">
+      <c r="N17" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="O17" s="47" t="s">
+      <c r="O17" s="9" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="18" spans="2:15" ht="15">
-      <c r="B18" s="3" t="s">
+      <c r="B18" s="34" t="s">
         <v>3</v>
       </c>
-      <c r="C18" s="4"/>
-      <c r="D18" s="15">
+      <c r="C18" s="35"/>
+      <c r="D18" s="36">
         <f>+F11</f>
         <v>0</v>
       </c>
-      <c r="E18" s="15"/>
-      <c r="G18" s="3" t="s">
+      <c r="E18" s="36"/>
+      <c r="G18" s="34" t="s">
         <v>9</v>
       </c>
-      <c r="H18" s="4"/>
-      <c r="I18" s="4"/>
-      <c r="J18" s="26">
+      <c r="H18" s="35"/>
+      <c r="I18" s="35"/>
+      <c r="J18" s="28">
         <v>450</v>
       </c>
-      <c r="K18" s="27"/>
-      <c r="L18" s="5"/>
-      <c r="M18" s="21" t="s">
+      <c r="K18" s="29"/>
+      <c r="M18" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="N18" s="22"/>
-      <c r="O18" s="48"/>
+      <c r="N18" s="5"/>
+      <c r="O18" s="10"/>
     </row>
     <row r="19" spans="2:15" ht="15">
-      <c r="B19" s="3" t="s">
+      <c r="B19" s="34" t="s">
         <v>4</v>
       </c>
-      <c r="C19" s="4"/>
-      <c r="D19" s="15">
+      <c r="C19" s="35"/>
+      <c r="D19" s="36">
         <f>+F12</f>
         <v>0</v>
       </c>
-      <c r="E19" s="15"/>
-      <c r="G19" s="3" t="s">
+      <c r="E19" s="36"/>
+      <c r="G19" s="34" t="s">
         <v>10</v>
       </c>
-      <c r="H19" s="4"/>
-      <c r="I19" s="4"/>
-      <c r="J19" s="24">
+      <c r="H19" s="35"/>
+      <c r="I19" s="35"/>
+      <c r="J19" s="30">
         <v>200</v>
       </c>
-      <c r="K19" s="25"/>
-      <c r="L19" s="5"/>
-      <c r="M19" s="21" t="s">
+      <c r="K19" s="31"/>
+      <c r="M19" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="N19" s="22"/>
-      <c r="O19" s="48"/>
+      <c r="N19" s="5"/>
+      <c r="O19" s="10"/>
     </row>
     <row r="20" spans="2:15" ht="15">
-      <c r="B20" s="18" t="s">
+      <c r="B20" s="23" t="s">
         <v>11</v>
       </c>
-      <c r="C20" s="19"/>
-      <c r="D20" s="20">
+      <c r="C20" s="37"/>
+      <c r="D20" s="38">
         <f>SUM(D18:E19)</f>
         <v>0</v>
       </c>
-      <c r="E20" s="18"/>
-      <c r="G20" s="3" t="s">
+      <c r="E20" s="23"/>
+      <c r="G20" s="34" t="s">
         <v>12</v>
       </c>
-      <c r="H20" s="4"/>
-      <c r="I20" s="4"/>
-      <c r="J20" s="24">
+      <c r="H20" s="35"/>
+      <c r="I20" s="35"/>
+      <c r="J20" s="30">
         <v>150</v>
       </c>
-      <c r="K20" s="25"/>
-      <c r="L20" s="5"/>
-      <c r="M20" s="18" t="s">
+      <c r="K20" s="31"/>
+      <c r="M20" s="23" t="s">
         <v>29</v>
       </c>
-      <c r="N20" s="18"/>
-      <c r="O20" s="49"/>
+      <c r="N20" s="23"/>
+      <c r="O20" s="11"/>
     </row>
     <row r="21" spans="2:15" ht="15">
-      <c r="G21" s="18" t="s">
+      <c r="G21" s="23" t="s">
         <v>13</v>
       </c>
-      <c r="H21" s="18"/>
-      <c r="I21" s="18"/>
-      <c r="J21" s="23">
+      <c r="H21" s="23"/>
+      <c r="I21" s="23"/>
+      <c r="J21" s="32">
         <f>SUM(J18:K19)</f>
         <v>650</v>
       </c>
-      <c r="K21" s="44"/>
+      <c r="K21" s="33"/>
     </row>
     <row r="25" spans="2:15" ht="15">
-      <c r="B25" s="10" t="s">
+      <c r="B25" s="24" t="s">
         <v>30</v>
       </c>
-      <c r="C25" s="10"/>
-      <c r="D25" s="10"/>
-      <c r="E25" s="10"/>
+      <c r="C25" s="24"/>
+      <c r="D25" s="24"/>
+      <c r="E25" s="24"/>
     </row>
     <row r="27" spans="2:15">
-      <c r="B27" s="50" t="s">
+      <c r="B27" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="C27" s="50" t="s">
+      <c r="C27" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="D27" s="50" t="s">
+      <c r="D27" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="E27" s="50" t="s">
+      <c r="E27" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="F27" s="51" t="s">
+      <c r="F27" s="18" t="s">
         <v>33</v>
       </c>
-      <c r="G27" s="51"/>
-      <c r="H27" s="51" t="s">
+      <c r="G27" s="18"/>
+      <c r="H27" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="I27" s="51"/>
-      <c r="J27" s="51" t="s">
+      <c r="I27" s="18"/>
+      <c r="J27" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="K27" s="51"/>
-      <c r="L27" s="51" t="s">
+      <c r="K27" s="18"/>
+      <c r="L27" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="M27" s="51"/>
-      <c r="N27" s="50" t="s">
+      <c r="M27" s="18"/>
+      <c r="N27" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="O27" s="50" t="s">
+      <c r="O27" s="12" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="28" spans="2:15" ht="15">
-      <c r="B28" s="52">
+      <c r="B28" s="13">
         <v>46196</v>
       </c>
-      <c r="C28" s="55">
+      <c r="C28" s="14">
         <v>0.43055555555555558</v>
       </c>
-      <c r="D28" s="55">
+      <c r="D28" s="14">
         <v>0.43263888888888891</v>
       </c>
-      <c r="E28" s="56" t="s">
+      <c r="E28" s="15" t="s">
         <v>36</v>
       </c>
-      <c r="F28" s="57" t="s">
+      <c r="F28" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="G28" s="58"/>
-      <c r="H28" s="53" t="s">
+      <c r="G28" s="17"/>
+      <c r="H28" s="19" t="s">
         <v>37</v>
       </c>
-      <c r="I28" s="54"/>
-      <c r="J28" s="59" t="s">
+      <c r="I28" s="20"/>
+      <c r="J28" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="K28" s="60"/>
-      <c r="L28" s="57">
+      <c r="K28" s="22"/>
+      <c r="L28" s="16">
         <v>200</v>
       </c>
-      <c r="M28" s="58"/>
-      <c r="N28" s="56">
+      <c r="M28" s="17"/>
+      <c r="N28" s="15">
         <v>2232</v>
       </c>
-      <c r="O28" s="55">
+      <c r="O28" s="14">
         <f>D28-C28</f>
         <v>2.0833333333333259E-3</v>
       </c>
     </row>
     <row r="29" spans="2:15" ht="15">
-      <c r="B29" s="52">
+      <c r="B29" s="13">
         <v>46196</v>
       </c>
-      <c r="C29" s="55">
+      <c r="C29" s="14">
         <v>0.45416666666666666</v>
       </c>
-      <c r="D29" s="55">
+      <c r="D29" s="14">
         <v>0.45833333333333331</v>
       </c>
-      <c r="E29" s="56" t="s">
+      <c r="E29" s="15" t="s">
         <v>36</v>
       </c>
-      <c r="F29" s="57" t="s">
+      <c r="F29" s="16" t="s">
         <v>9</v>
       </c>
-      <c r="G29" s="58"/>
-      <c r="H29" s="53" t="s">
+      <c r="G29" s="17"/>
+      <c r="H29" s="19" t="s">
         <v>37</v>
       </c>
-      <c r="I29" s="54"/>
-      <c r="J29" s="59" t="s">
+      <c r="I29" s="20"/>
+      <c r="J29" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="K29" s="60"/>
-      <c r="L29" s="57">
+      <c r="K29" s="22"/>
+      <c r="L29" s="16">
         <v>450</v>
       </c>
-      <c r="M29" s="58"/>
-      <c r="N29" s="56">
+      <c r="M29" s="17"/>
+      <c r="N29" s="15">
         <v>2233</v>
       </c>
-      <c r="O29" s="55">
+      <c r="O29" s="14">
         <f t="shared" ref="O29:O30" si="0">D29-C29</f>
         <v>4.1666666666666519E-3</v>
       </c>
     </row>
     <row r="30" spans="2:15" ht="15">
-      <c r="B30" s="52">
+      <c r="B30" s="13">
         <v>46196</v>
       </c>
-      <c r="C30" s="55">
+      <c r="C30" s="14">
         <v>0.47499999999999998</v>
       </c>
-      <c r="D30" s="55">
+      <c r="D30" s="14">
         <v>0.47638888888888886</v>
       </c>
-      <c r="E30" s="56" t="s">
+      <c r="E30" s="15" t="s">
         <v>36</v>
       </c>
-      <c r="F30" s="57" t="s">
+      <c r="F30" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="G30" s="58"/>
-      <c r="H30" s="53" t="s">
+      <c r="G30" s="17"/>
+      <c r="H30" s="19" t="s">
         <v>37</v>
       </c>
-      <c r="I30" s="54"/>
-      <c r="J30" s="59" t="s">
+      <c r="I30" s="20"/>
+      <c r="J30" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="K30" s="60"/>
-      <c r="L30" s="57">
+      <c r="K30" s="22"/>
+      <c r="L30" s="16">
         <v>150</v>
       </c>
-      <c r="M30" s="58"/>
-      <c r="N30" s="56">
+      <c r="M30" s="17"/>
+      <c r="N30" s="15">
         <v>2234</v>
       </c>
-      <c r="O30" s="55">
+      <c r="O30" s="14">
         <f t="shared" si="0"/>
         <v>1.388888888888884E-3</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="63">
-    <mergeCell ref="L29:M29"/>
-    <mergeCell ref="L30:M30"/>
-    <mergeCell ref="F28:G28"/>
-    <mergeCell ref="F30:G30"/>
-    <mergeCell ref="F29:G29"/>
-    <mergeCell ref="L27:M27"/>
-    <mergeCell ref="H28:I28"/>
-    <mergeCell ref="H29:I29"/>
-    <mergeCell ref="H30:I30"/>
-    <mergeCell ref="J28:K28"/>
-    <mergeCell ref="J29:K29"/>
-    <mergeCell ref="J30:K30"/>
-    <mergeCell ref="L28:M28"/>
-    <mergeCell ref="M20:N20"/>
-    <mergeCell ref="B25:E25"/>
-    <mergeCell ref="F27:G27"/>
-    <mergeCell ref="H27:I27"/>
-    <mergeCell ref="J27:K27"/>
-    <mergeCell ref="M15:P15"/>
-    <mergeCell ref="J17:K17"/>
-    <mergeCell ref="J18:K18"/>
-    <mergeCell ref="J19:K19"/>
-    <mergeCell ref="J21:K21"/>
-    <mergeCell ref="G20:I20"/>
-    <mergeCell ref="J20:K20"/>
-    <mergeCell ref="G18:I18"/>
-    <mergeCell ref="G19:I19"/>
-    <mergeCell ref="G21:I21"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="D18:E18"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="D19:E19"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="D20:E20"/>
+    <mergeCell ref="B8:N8"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="D10:E10"/>
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="H10:I10"/>
+    <mergeCell ref="J10:K10"/>
+    <mergeCell ref="H11:I11"/>
+    <mergeCell ref="H12:I12"/>
+    <mergeCell ref="L10:M10"/>
+    <mergeCell ref="N10:O10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="D11:E11"/>
+    <mergeCell ref="J11:K11"/>
     <mergeCell ref="A1:O3"/>
     <mergeCell ref="D4:L5"/>
     <mergeCell ref="B15:E15"/>
@@ -2186,19 +2147,40 @@
     <mergeCell ref="D12:E12"/>
     <mergeCell ref="F11:G11"/>
     <mergeCell ref="F12:G12"/>
-    <mergeCell ref="H11:I11"/>
-    <mergeCell ref="H12:I12"/>
-    <mergeCell ref="L10:M10"/>
-    <mergeCell ref="N10:O10"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="D11:E11"/>
-    <mergeCell ref="J11:K11"/>
-    <mergeCell ref="B8:N8"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="D10:E10"/>
-    <mergeCell ref="F10:G10"/>
-    <mergeCell ref="H10:I10"/>
-    <mergeCell ref="J10:K10"/>
+    <mergeCell ref="G18:I18"/>
+    <mergeCell ref="G19:I19"/>
+    <mergeCell ref="G21:I21"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="D18:E18"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="D19:E19"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="D20:E20"/>
+    <mergeCell ref="M15:P15"/>
+    <mergeCell ref="J17:K17"/>
+    <mergeCell ref="J18:K18"/>
+    <mergeCell ref="J19:K19"/>
+    <mergeCell ref="J21:K21"/>
+    <mergeCell ref="J20:K20"/>
+    <mergeCell ref="M20:N20"/>
+    <mergeCell ref="B25:E25"/>
+    <mergeCell ref="F27:G27"/>
+    <mergeCell ref="H27:I27"/>
+    <mergeCell ref="J27:K27"/>
+    <mergeCell ref="G20:I20"/>
+    <mergeCell ref="L27:M27"/>
+    <mergeCell ref="H28:I28"/>
+    <mergeCell ref="H29:I29"/>
+    <mergeCell ref="H30:I30"/>
+    <mergeCell ref="J28:K28"/>
+    <mergeCell ref="J29:K29"/>
+    <mergeCell ref="J30:K30"/>
+    <mergeCell ref="L28:M28"/>
+    <mergeCell ref="L29:M29"/>
+    <mergeCell ref="L30:M30"/>
+    <mergeCell ref="F28:G28"/>
+    <mergeCell ref="F30:G30"/>
+    <mergeCell ref="F29:G29"/>
   </mergeCells>
   <conditionalFormatting sqref="H28:I30">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">

</xml_diff>